<commit_message>
Refactor PPC functions to auto-detect active _rep parameters
</commit_message>
<xml_diff>
--- a/documentation_files/documentation_tables.xlsx
+++ b/documentation_files/documentation_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/kale_bentley_dfw_wa_gov/Documents/Projects/Creel/GitHub/CreelEstimates/documentation_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="642" documentId="13_ncr:1_{06BDCB52-A10A-4652-9501-BAA58E581D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2F6D855-881A-4181-A9EC-550790DD7EBF}"/>
+  <xr:revisionPtr revIDLastSave="643" documentId="13_ncr:1_{06BDCB52-A10A-4652-9501-BAA58E581D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F94C43E3-70BC-4A08-82B5-986FCED8D7A6}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="2" xr2:uid="{D87A213F-20EA-453F-96F1-E2F9D588DE08}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D87A213F-20EA-453F-96F1-E2F9D588DE08}"/>
   </bookViews>
   <sheets>
     <sheet name="design_stratification" sheetId="7" r:id="rId1"/>
@@ -30,6 +30,9 @@
     <sheet name="PE_effort" sheetId="3" r:id="rId15"/>
     <sheet name="PE_catch" sheetId="8" r:id="rId16"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">YAML_parameters!$A$1:$D$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -975,9 +978,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1015,7 +1018,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1121,7 +1124,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1263,7 +1266,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2292,6 +2295,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D1" xr:uid="{3C534D12-2EFF-44CC-BEBB-F36901043652}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3341,4 +3345,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{45011977-b912-4387-97a4-f4c94a801377}" enabled="1" method="Standard" siteId="{11d0e217-264e-400a-8ba0-57dcc127d72d}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>